<commit_message>
Update carousel-log.xlsx after carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,7 +623,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>7</v>
       </c>
@@ -880,6 +879,391 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>Blog post carousel - ties to Step Up or Step Out</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>The Brilliant Jerk Problem</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/handle-brilliant-jerk-work</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/brilliant-jerk-problem-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Recognise the Real Cost</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/handle-brilliant-jerk-work</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/recognise-the-real-cost-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Diagnose Before You Act</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/handle-brilliant-jerk-work</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/diagnose-before-you-act-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Intervene With Structure</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/handle-brilliant-jerk-work</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/intervene-with-structure-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Reinforce Culture Through Action</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/handle-brilliant-jerk-work</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/reinforce-culture-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>6 Mistakes Leaders Make With Brilliant Jerks</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/handle-brilliant-jerk-work</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/6-mistakes-brilliant-jerks-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Your First 30 Days Action Plan</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/handle-brilliant-jerk-work</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/30-day-action-plan-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Blog post carousel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after testimonial+service posts
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1267,6 +1267,116 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Testimonial: Edward Amey - Best Offsite</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://consultclarity.org/testimonials</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/testimonial-edward-amey-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Client testimonial carousel - Edward Amey, USA, leadership offsite</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Service: The Human Side of AI in Schools</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://consultclarity.org</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/service-ai-keynote-schools-2026-03-24</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Service niche carousel - AI keynote for schools</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after carousel run 2026-03-25
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2202,6 +2202,363 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>decision-fatigue-intro</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leadership-decision-fatigue</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>8</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/jonno-alt/social-images/main/carousels/decision-fatigue-intro-2026-03-25/</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>TikTok, YouTube, Pinterest</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>decision-architecture</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leadership-decision-fatigue</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/jonno-alt/social-images/main/carousels/decision-architecture-2026-03-25/</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>TikTok, YouTube, Pinterest</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>meeting-design</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leadership-decision-fatigue</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/jonno-alt/social-images/main/carousels/meeting-design-2026-03-25/</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>TikTok, YouTube, Pinterest</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>energy-management</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leadership-decision-fatigue</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>8</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/jonno-alt/social-images/main/carousels/energy-management-2026-03-25/</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>TikTok, YouTube, Pinterest</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>cognitive-load-reduction</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leadership-decision-fatigue</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>7</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/jonno-alt/social-images/main/carousels/cognitive-load-reduction-2026-03-25/</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>TikTok, YouTube, Pinterest</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>team-structure-decisions</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leadership-decision-fatigue</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>8</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/jonno-alt/social-images/main/carousels/team-structure-decisions-2026-03-25/</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>PENDING (Buffer rate limit)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>TikTok, YouTube, Pinterest</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>decision-fatigue-mistakes</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leadership-decision-fatigue</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>8</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/jonno-alt/social-images/main/carousels/decision-fatigue-mistakes-2026-03-25/</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>PENDING (Buffer rate limit)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>TikTok, YouTube, Pinterest</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after Steps After Working Genius carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2772,6 +2772,281 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Your First Week After Working Genius</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/steps-after-working-genius</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>7</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/first-week-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards configured)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Steps After Working Genius blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Month One: Build the Foundation</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/steps-after-working-genius</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>8</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/month-one-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards configured)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Steps After Working Genius blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Redesign How Your Team Works</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/steps-after-working-genius</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>8</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/redesign-work-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards configured)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Steps After Working Genius blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Make Working Genius Stick</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/steps-after-working-genius</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>8</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/make-it-stick-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards configured)</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Steps After Working Genius blog post carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Build a Working Genius Culture</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/steps-after-working-genius</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>7</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/genius-culture-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards configured)</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Steps After Working Genius blog post carousel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after WG-Hiring carousel run 2026-03-25
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3047,6 +3047,556 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>wg-hiring-foundation</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>7</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-foundation/</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Understanding the Foundation (Tips 1-5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>wg-hiring-diagnosis</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>7</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-diagnosis/</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Diagnosing Your Team Before Hiring (Tips 6-10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>wg-hiring-job-descriptions</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>7</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-job-descriptions/</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Rewriting Job Descriptions (Tips 11-15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>wg-hiring-interviews</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>7</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-interviews/</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Designing the Interview Process (Tips 16-20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>wg-hiring-assessment</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>7</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-assessment/</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Using the Assessment Strategically (Tips 21-25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>wg-hiring-decisions</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>7</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-decisions/</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Making the Hiring Decision (Tips 26-30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>wg-hiring-onboarding</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>7</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-onboarding/</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Onboarding With Working Genius (Tips 31-35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>wg-hiring-mistakes</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>7</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-mistakes/</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Common Hiring Mistakes to Avoid (Tips 36-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>wg-hiring-advanced</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>7</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-advanced/</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Advanced Hiring Strategies (Tips 41-45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>wg-hiring-measuring</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/working-genius-for-hiring</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>7</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-hiring-2026-03-25/wg-hiring-measuring/</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Instagram photo tag verification</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Measuring Success After Hiring (Tips 46-50)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after sleep-leadership carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3597,6 +3597,391 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>sleep-leadership-stats</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/how-sleep-affects-leadership</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>8</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/sleep-leadership-stats-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube (Mar 30)</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Blog post carousel - How Sleep Affects Leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>sleep-protect-your-window</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/how-sleep-affects-leadership</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>6</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/sleep-protect-your-window-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube (Mar 30)</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Blog post carousel - How Sleep Affects Leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>sleep-manage-your-inputs</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/how-sleep-affects-leadership</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>6</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/sleep-manage-your-inputs-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube (Mar 30)</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Blog post carousel - How Sleep Affects Leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>sleep-environment-and-light</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/how-sleep-affects-leadership</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>8</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/sleep-environment-and-light-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube (Mar 30)</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Blog post carousel - How Sleep Affects Leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>sleep-stress-and-rumination</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/how-sleep-affects-leadership</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>6</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/sleep-stress-and-rumination-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube (Mar 30)</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Blog post carousel - How Sleep Affects Leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>sleep-culture-and-recovery</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/how-sleep-affects-leadership</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>8</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/sleep-culture-and-recovery-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube (Mar 30)</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Blog post carousel - How Sleep Affects Leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>sleep-mistakes-leaders-make</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/how-sleep-affects-leadership</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>7</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/sleep-mistakes-leaders-make-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube (Mar 31)</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Blog post carousel - How Sleep Affects Leadership</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after loneliness carousel run 2026-03-25
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3982,6 +3982,363 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>loneliness-external-support</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/overcome-loneliness-at-the-top</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>7</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/loneliness-external-support-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, YouTube, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions, Instagram verify tags, Facebook personal tags, TikTok captions</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>loneliness-honest-culture</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/overcome-loneliness-at-the-top</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>7</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/loneliness-honest-culture-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, YouTube, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions, Instagram verify tags, Facebook personal tags, TikTok captions</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>loneliness-unique-pressures</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/overcome-loneliness-at-the-top</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>7</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/loneliness-unique-pressures-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, YouTube, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions, Instagram verify tags, Facebook personal tags, TikTok captions</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>loneliness-personal-wellbeing</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/overcome-loneliness-at-the-top</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>7</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/loneliness-personal-wellbeing-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, YouTube, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions, Instagram verify tags, Facebook personal tags, TikTok captions</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>loneliness-daily-habits</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/overcome-loneliness-at-the-top</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>7</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/loneliness-daily-habits-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, YouTube, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions, Instagram verify tags, Facebook personal tags, TikTok captions</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>loneliness-mistakes</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/overcome-loneliness-at-the-top</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>7</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/loneliness-mistakes-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, YouTube, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions, Instagram verify tags, Facebook personal tags, TikTok captions</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>loneliness-30-day-plan</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/overcome-loneliness-at-the-top</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>7</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/loneliness-30-day-plan-2026-03-25</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, YouTube, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions, Instagram verify tags, Facebook personal tags, TikTok captions</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after caring-hurts-leadership run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4031,7 +4031,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4082,7 +4081,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4133,7 +4131,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4184,7 +4181,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4235,7 +4231,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4286,7 +4281,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4337,7 +4331,226 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Why Caring Too Much Hurts</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/caring-hurts-leadership</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>8</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/caring-hurts-leadership-2026-03-25/why-caring-hurts</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, Facebook personal profile tags, YouTube @mention editing</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Blog post carousel. Pinterest skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Signs 1-5: Caring Hurts Leadership</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/caring-hurts-leadership</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>7</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/caring-hurts-leadership-2026-03-25/signs-1-to-5</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, Facebook personal profile tags, YouTube @mention editing</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Blog post carousel. Pinterest skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Signs 6-10: Caring Hurts Leadership</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/caring-hurts-leadership</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>7</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/caring-hurts-leadership-2026-03-25/signs-6-to-10</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, Facebook personal profile tags, YouTube @mention editing</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Blog post carousel. Pinterest skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>From Caring That Hurts to Caring That Builds</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/caring-hurts-leadership</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>8</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/caring-hurts-leadership-2026-03-25/caring-that-builds</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, Facebook personal profile tags, YouTube @mention editing</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Blog post carousel. Pinterest skipped.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after Leaders Eat Last carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4552,6 +4552,226 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Why Read Leaders Eat Last</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>8</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/leaders-eat-last-2026-03-26/why-read-leaders-eat-last</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Leaders Eat Last book rec series</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>The Circle of Safety</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>8</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/leaders-eat-last-2026-03-26/circle-of-safety</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Leaders Eat Last book rec series</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>The 4 Chemicals of Leadership</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>8</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/leaders-eat-last-2026-03-26/four-chemicals-of-leadership</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Leaders Eat Last book rec series</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Key Lessons from Leaders Eat Last</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>8</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/leaders-eat-last-2026-03-26/key-lessons-leaders-eat-last</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>X/Twitter photo tags, YouTube @mentions</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Leaders Eat Last book rec series</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after carousel run - Craig Groeschel Podcast
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K84"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4922,6 +4922,171 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Why Listen to Craig Groeschel</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>N/A - Podcast Rec</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>8</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/craig-groeschel-podcast-2026-03-26/why-listen</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>X photo tags, YT @mentions</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Yes (pin created but Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Pinterest skipped. TikTok scheduled Mar 31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>5 Key Themes from Craig Groeschel</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>N/A - Podcast Rec</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>7</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/craig-groeschel-podcast-2026-03-26/key-themes</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>X photo tags, YT @mentions</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Yes (pin created but Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Pinterest skipped. TikTok scheduled Mar 31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>3 Reasons to Subscribe</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>N/A - Podcast Rec</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>6</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/craig-groeschel-podcast-2026-03-26/reasons-subscribe</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>X photo tags, YT @mentions</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Yes (pin created but Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Pinterest skipped. TikTok scheduled Mar 31.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after ASBA testimonial carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5087,6 +5087,156 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>asba-working-genius-in-action</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>7</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asba-working-genius-in-action-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ASBA 2025 testimonial carousel. TikTok/YouTube hit Buffer daily creation limits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>asba-93-percent-rated-excellent</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>7</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asba-93-percent-rated-excellent-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ASBA 2025 testimonial carousel. TikTok/YouTube hit Buffer daily creation limits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>asba-what-school-leaders-took-away</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>7</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asba-what-school-leaders-took-away-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>TikTok (daily limit), YouTube (daily limit), Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ASBA 2025 testimonial carousel. TikTok/YouTube hit Buffer daily creation limits.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after carousel run - offsite corporates
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5237,6 +5237,226 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>offsite-why-your-team-needs-one</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Service page: Leadership Team Offsite for Corporates</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>8</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/offsite-why-your-team-needs-one-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>N/A - service post</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>N/A - no boards</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Service promotion carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>offsite-what-to-expect</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Service page: Leadership Team Offsite for Corporates</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>8</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/offsite-what-to-expect-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>N/A - service post</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>N/A - no boards</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Service promotion carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>offsite-common-mistakes</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Service page: Leadership Team Offsite for Corporates</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>8</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/offsite-common-mistakes-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>N/A - service post</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>N/A - no boards</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Service promotion carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>offsite-book-your-offsite</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Service page: Leadership Team Offsite for Corporates</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>7</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/offsite-book-your-offsite-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>N/A - service post</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>N/A - no boards</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Service promotion carousel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log after Topic 1
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K94"/>
+  <dimension ref="A1:K98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5457,6 +5457,226 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>5-dysfunctions-overview</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>N/A (Framework topic)</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>9</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Framework explainer carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>5-dysfunctions-trust-conflict</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>N/A (Framework topic)</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>8</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Framework explainer carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>5-dysfunctions-commitment-results</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>N/A (Framework topic)</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>9</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Framework explainer carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>5-dysfunctions-action-plan</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>N/A (Framework topic)</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>8</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Framework explainer carousel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after Topic 2
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K98"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5677,6 +5677,171 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>imposter-syndrome-signs</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>N/A (Blog topic)</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>8</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/imposter-syndrome-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Blog topic carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>imposter-syndrome-cost</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>N/A (Blog topic)</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>8</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/imposter-syndrome-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Blog topic carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>imposter-syndrome-overcome</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>N/A (Blog topic)</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>8</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/imposter-syndrome-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Blog topic carousel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after Topic 3
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5842,6 +5842,171 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>unreasonable-hospitality-why-read</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>7</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/unreasonable-hospitality-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Book rec carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>unreasonable-hospitality-lessons</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>7</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/unreasonable-hospitality-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Book rec carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>unreasonable-hospitality-apply</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>7</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/unreasonable-hospitality-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Book rec carousel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - session complete (4 topics)
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K104"/>
+  <dimension ref="A1:K107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6007,6 +6007,171 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>losing-teachers-warning-signs</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>N/A (Pain Point)</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>8</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/losing-good-teachers-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Pain point carousel - school topic</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>losing-teachers-real-reasons</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>N/A (Pain Point)</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>8</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/losing-good-teachers-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Pain point carousel - school topic</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>losing-teachers-what-to-do</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>N/A (Pain Point)</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>7</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/losing-good-teachers-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Pain point carousel - school topic</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update after Topic 1: HBR IdeaCast
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6172,6 +6172,141 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>hbr-ideacast-why-listen</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>8</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/hbr-ideacast-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Podcast rec: HBR IdeaCast</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>hbr-ideacast-key-themes</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>7</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/hbr-ideacast-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Podcast rec: HBR IdeaCast</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>hbr-ideacast-reasons-subscribe</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>6</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/hbr-ideacast-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Podcast rec: HBR IdeaCast</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 2 Redlands College
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K110"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6307,6 +6307,171 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>redlands-wg-overview</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Testimonial: Michael Quach, Redlands College</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>7</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/redlands-working-genius-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Actual testimonial quote not found online - built around verified Redlands College engagement facts</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>redlands-wg-discoveries</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Testimonial: Michael Quach, Redlands College</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>7</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/redlands-working-genius-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Actual testimonial quote not found online - built around verified Redlands College engagement facts</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>redlands-wg-book-session</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Testimonial: Michael Quach, Redlands College</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>6</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/redlands-working-genius-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Actual testimonial quote not found online - built around verified Redlands College engagement facts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 3 Schools WG
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6472,6 +6472,159 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>schools-wg-why</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Service: Working Genius Workshop for Schools</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>7</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/schools-working-genius-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>schools-wg-how</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Service: Working Genius Workshop for Schools</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>6</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/schools-working-genius-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>schools-wg-transform</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Service: Working Genius Workshop for Schools</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>6</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/schools-working-genius-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 4 WG Session
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:K119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6521,7 +6521,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6572,7 +6571,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6623,7 +6621,159 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>wg-session-inside</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>What Actually Happens in a Working Genius Session</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>7</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-session-inside-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>wg-session-moments</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>What Actually Happens in a Working Genius Session</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>7</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-session-inside-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>wg-session-book</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>What Actually Happens in a Working Genius Session</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>5</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/wg-session-inside-2026-03-26</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>

</xml_diff>

<commit_message>
Update carousel log - Leading Through Uncertainty
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K119"/>
+  <dimension ref="A1:K123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6671,7 +6671,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6722,7 +6721,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6773,7 +6771,226 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>understanding-uncertainty</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leading-through-uncertainty</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>8</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/leading-through-uncertainty-2026-03-26/understanding-uncertainty</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>All platforms scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>decision-making-uncertainty</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leading-through-uncertainty</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>8</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/leading-through-uncertainty-2026-03-26/decision-making-uncertainty</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>All platforms scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>communication-trust-uncertainty</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leading-through-uncertainty</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>8</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/leading-through-uncertainty-2026-03-26/communication-trust-uncertainty</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>All platforms scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>resilience-adaptive-strategy</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/leading-through-uncertainty</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>8</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/leading-through-uncertainty-2026-03-26/resilience-adaptive-strategy</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>All platforms scheduled</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>

</xml_diff>

<commit_message>
Update - Topic 2 Radical Candor
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K123"/>
+  <dimension ref="A1:K126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6992,6 +6992,171 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>radical-candor-why-read</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>8</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/radical-candor-2026-03-26/radical-candor-why-read</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>All platforms scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>radical-candor-four-quadrants</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>8</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/radical-candor-2026-03-26/radical-candor-four-quadrants</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>All platforms scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>radical-candor-in-practice</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>N/A (Book Rec)</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>8</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/radical-candor-2026-03-26/radical-candor-in-practice</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>All platforms scheduled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel log after Topic 1
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K126"/>
+  <dimension ref="A1:K129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7157,6 +7157,171 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>why-priorities-fail</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>N/A - Pain Point</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>8</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/priorities-same-things-2026-03-26/why-priorities-fail</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Pain point topic, no people to tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>signs-plan-will-fail</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>N/A - Pain Point</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>7</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/priorities-same-things-2026-03-26/signs-plan-will-fail</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Pain point topic, no people to tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>break-the-cycle</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>N/A - Pain Point</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>8</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/priorities-same-things-2026-03-26/break-the-cycle</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>IG, GBP, TikTok, YT (LI/FB/Threads/X/Bluesky failed)</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>LI, FB, Threads, X, Bluesky</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Pain point topic, no people to tag</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log: Add worklife-podcast-rec + worklife-why-listen
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K129"/>
+  <dimension ref="A1:K131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7322,6 +7322,108 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>worklife-podcast-rec</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://www.yourthoughtpartner.com/blog/worklife-with-adam-grant-podcast</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>8</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/worklife-adam-grant-2026-03-26/worklife-podcast-rec</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Founder, Clarity Group Global</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>All 9 platforms scheduled. @adamgrant tagged on Instagram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>worklife-why-listen</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://www.yourthoughtpartner.com/blog/worklife-with-adam-grant-podcast</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>7</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/worklife-adam-grant-2026-03-26/worklife-why-listen</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Founder, Clarity Group Global</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>All 9 platforms scheduled. 5 Reasons Leaders Should Listen theme.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log: Add keynote-speaking + exec-dysfunction carousels
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:K135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7351,7 +7351,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
           <t>Founder, Clarity Group Global</t>
@@ -7402,7 +7401,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr">
         <is>
           <t>Founder, Clarity Group Global</t>
@@ -7421,6 +7419,194 @@
       <c r="K131" t="inlineStr">
         <is>
           <t>All 9 platforms scheduled. 5 Reasons Leaders Should Listen theme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>keynote-speaking-service</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr"/>
+      <c r="D132" t="n">
+        <v>8</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/keynote-speaking-2026-03-26/keynote-speaking-service</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Founder, Clarity Group Global</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>6 keynote topics overview. All 9 platforms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>why-book-jonno</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr"/>
+      <c r="D133" t="n">
+        <v>7</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/keynote-speaking-2026-03-26/why-book-jonno</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Founder, Clarity Group Global</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>5 reasons to book Jonno. All 9 platforms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>exec-team-dysfunction</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="n">
+        <v>9</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/exec-team-dysfunction-2026-03-26/exec-team-dysfunction</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Founder, Clarity Group Global</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>7 signs of dysfunction. Lencioni framework. All 9 platforms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="n">
+        <v>7</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/exec-team-dysfunction-2026-03-26/fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Founder, Clarity Group Global</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>5 steps to high performance. Lencioni framework. All 9 platforms.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update carousel log - Topic 1 ASBA proof
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K135"/>
+  <dimension ref="A1:K137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7433,7 +7433,6 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr"/>
       <c r="D132" t="n">
         <v>8</v>
       </c>
@@ -7447,7 +7446,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
           <t>Founder, Clarity Group Global</t>
@@ -7480,7 +7478,6 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
       <c r="D133" t="n">
         <v>7</v>
       </c>
@@ -7494,7 +7491,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
           <t>Founder, Clarity Group Global</t>
@@ -7527,7 +7523,6 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
       <c r="D134" t="n">
         <v>9</v>
       </c>
@@ -7541,7 +7536,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
           <t>Founder, Clarity Group Global</t>
@@ -7574,7 +7568,6 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
       <c r="D135" t="n">
         <v>7</v>
       </c>
@@ -7588,7 +7581,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr">
         <is>
           <t>Founder, Clarity Group Global</t>
@@ -7607,6 +7599,106 @@
       <c r="K135" t="inlineStr">
         <is>
           <t>5 steps to high performance. Lencioni framework. All 9 platforms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>asba-93-percent-proof</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>8</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asba-93-percent-proof-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>YouTube (disconnected), Google Business (disconnected)</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Stats/proof topic about ASBA 2025 conference results</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>asba-what-makes-pd-great</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>8</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/asba-what-makes-pd-great-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>YouTube (disconnected), Google Business (disconnected)</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>5 reasons Working Genius PD stands out</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update carousel log - Topic 2
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K137"/>
+  <dimension ref="A1:K140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7702,6 +7702,156 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>extreme-ownership-why-read</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>8</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/extreme-ownership-why-read-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>LI,FB,IG,Threads,X,Bluesky,TikTok</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>YouTube,GBP (disconnected)</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Why read Extreme Ownership</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>extreme-ownership-principles</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>8</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/extreme-ownership-principles-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>LI,FB,IG,Threads,X,Bluesky,TikTok</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>YouTube,GBP (disconnected)</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>5 key principles</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>extreme-ownership-apply</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>7</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/extreme-ownership-apply-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>LI,FB,IG,Threads,X,Bluesky,TikTok</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>YouTube,GBP (disconnected)</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>How to apply</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log - Topic 3 meeting perfect
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K140"/>
+  <dimension ref="A1:K142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7852,6 +7852,106 @@
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>perfect-meeting-danger</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>8</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/perfect-meeting-danger-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>YouTube, Google Business</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Pain point topic, no people to tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>perfect-meeting-fix</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>8</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/perfect-meeting-fix-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>YouTube, Google Business</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Pain point topic, no people to tag</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log - Topic 4 Learning Leader
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K142"/>
+  <dimension ref="A1:K144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7952,6 +7952,106 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>learning-leader-rec</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>8</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/learning-leader-rec-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>YouTube, Google Business</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Podcast recommendation overview, tags @ryanhawk12</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>learning-leader-lessons</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>8</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/learning-leader-lessons-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>YouTube, Google Business</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>5 leadership lessons from the show, tags @ryanhawk12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 1: Edward Amey testimonial
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -59,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K144"/>
+  <dimension ref="A1:K146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8052,6 +8055,102 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>offsite-insights-edward-amey</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D145" t="n">
+        <v>8</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/testimonial-edward-amey-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Testimonial topic. Content from EP225 podcast and public bio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>leadership-disability-edward-amey</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D146" t="n">
+        <v>7</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/testimonial-edward-amey-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Testimonial topic. Content from EP225 podcast and public bio.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 2: Executive Coaching
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K146"/>
+  <dimension ref="A1:K149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8151,6 +8151,150 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>why-leaders-need-a-coach</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D147" t="n">
+        <v>8</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/service-executive-coaching-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Leadership Coach | Author</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Service promo: Executive Coaching for Leaders</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>what-coaching-looks-like</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D148" t="n">
+        <v>8</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/service-executive-coaching-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Leadership Coach | Author</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Service promo: Executive Coaching for Leaders</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>cost-of-no-coach</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="D149" t="n">
+        <v>8</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/service-executive-coaching-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Leadership Coach | Author</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Service promo: Executive Coaching for Leaders</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 1 Working Genius
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K149"/>
+  <dimension ref="A1:K152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8295,6 +8295,171 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>wg-6-types</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>N/A - Framework topic</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>8</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/working-genius-6-types-2026-03-27/wg-6-types</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Working Genius: 6 Types Explained</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>wg-genius-or-frustration</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>N/A - Framework topic</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>8</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/working-genius-6-types-2026-03-27/wg-genius-or-frustration</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Genius, Competency, or Frustration</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>wg-transforms-teams</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>N/A - Framework topic</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>8</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/working-genius-6-types-2026-03-27/wg-transforms-teams</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>How Working Genius Transforms Teams</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 2 Five Dysfunctions
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K152"/>
+  <dimension ref="A1:K155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8460,6 +8460,171 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>5d-overview</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>N/A - Book summary</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>8</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-team-2026-03-27/5d-overview</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>All 9 platforms</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Five Dysfunctions Overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>5d-overcome</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>N/A - Book summary</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>8</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-team-2026-03-27/5d-overcome</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>All 9 platforms</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>How to Overcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>5d-warning-signs</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>N/A - Book summary</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>8</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/five-dysfunctions-team-2026-03-27/5d-warning-signs</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>All 9 platforms</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Warning Signs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel log - Crucial Conversations
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K155"/>
+  <dimension ref="A1:K158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8625,6 +8625,141 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>crucial-conversations-why-read</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>8</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/crucial-conversations-book-rec-2026-03-27/crucial-conversations-why-read</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Book rec carousel. No people tagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>crucial-conversations-7-skills</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>9</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/crucial-conversations-book-rec-2026-03-27/crucial-conversations-7-skills</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Book rec carousel. No people tagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>crucial-conversations-apply</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>8</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/crucial-conversations-book-rec-2026-03-27/crucial-conversations-apply</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Book rec carousel. No people tagged.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel log - Board Offsite Nonprofits
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K163"/>
+  <dimension ref="A1:K165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8985,6 +8985,96 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>board-offsite-why</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>8</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/board-offsite-nonprofits-2026-03-27/board-offsite-why</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Service carousel for Board Offsite for Nonprofits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>board-offsite-5-signs</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>7</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/board-offsite-nonprofits-2026-03-27/board-offsite-5-signs</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Service carousel for Board Offsite for Nonprofits.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel log - Topic 1 pre-brief
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K165"/>
+  <dimension ref="A1:K167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9075,6 +9075,106 @@
         </is>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>The Pre-Brief Call</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>8</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/pre-brief-zoom-call-2026-03-27/pre-brief-call</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Behind the scenes carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>5 Questions Before Every Offsite</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>8</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/pre-brief-zoom-call-2026-03-27/5-questions-before-offsite</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Behind the scenes carousel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel log - Topic 2 VBT
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K167"/>
+  <dimension ref="A1:K170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9175,6 +9175,171 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>What Is Vulnerability-Based Trust?</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>8</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/vulnerability-based-trust-2026-03-27/what-is-vulnerability-based-trust</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Concept overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>7 Ways to Build Vulnerability-Based Trust</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>9</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/vulnerability-based-trust-2026-03-27/7-ways-vulnerability-trust</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Practical tips</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>The Leader Must Go First</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>8</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/vulnerability-based-trust-2026-03-27/leader-must-go-first</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Leadership role in trust</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update - Topic 3 Atomic Habits
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K170"/>
+  <dimension ref="A1:K172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9340,6 +9340,106 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Why Every Leader Should Read Atomic Habits</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>8</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/atomic-habits-2026-03-27/atomic-habits-book-rec</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Book rec carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>The 4 Laws of Behaviour Change</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>8</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/atomic-habits-2026-03-27/4-laws-behaviour-change</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>Book rec carousel - framework</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx after Topic 1
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K172"/>
+  <dimension ref="A1:K174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9440,6 +9440,100 @@
         </is>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>offsite-why-nothing-changed</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Pain Point: We Did an Offsite and Nothing Changed</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>8</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/offsite-pain-point-2026-03-27/offsite-why-nothing-changed</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>offsite-how-to-stick</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Pain Point: We Did an Offsite and Nothing Changed</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>8</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/offsite-pain-point-2026-03-27/offsite-how-to-stick</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log: 2 Maxwell Podcast entries
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K174"/>
+  <dimension ref="A1:K176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9469,7 +9469,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
-      <c r="G173" t="inlineStr"/>
       <c r="H173" t="inlineStr">
         <is>
           <t>Leadership Team Facilitator | Author</t>
@@ -9485,7 +9484,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -9516,7 +9514,6 @@
           <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr"/>
       <c r="H174" t="inlineStr">
         <is>
           <t>Leadership Team Facilitator | Author</t>
@@ -9532,7 +9529,116 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>maxwell-podcast-why-listen</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>N/A (Podcast Rec)</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>8</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/maxwell-podcast-2026-03-27/maxwell-podcast-why-listen</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Podcast recommendation carousel - Why Listen</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>maxwell-podcast-key-themes</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>N/A (Podcast Rec)</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>8</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/maxwell-podcast-2026-03-27/maxwell-podcast-key-themes</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Podcast recommendation carousel - Key Themes</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>

</xml_diff>

<commit_message>
Update carousel-log: Topic 3 Strategic Planning
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K176"/>
+  <dimension ref="A1:K178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9640,6 +9640,116 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>strategic-plan-why-facilitator</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>N/A (Service)</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>8</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/strategic-plan-2026-03-27/strategic-plan-why-facilitator</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Strategic Planning Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Service carousel - Why You Need a Facilitator</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>strategic-plan-5-signs-dust</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>N/A (Service)</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>8</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/strategic-plan-2026-03-27/strategic-plan-5-signs-dust</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Strategic Planning Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Service carousel - 5 Signs Plan Gathering Dust</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Final update: 8 carousels logged
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K178"/>
+  <dimension ref="A1:K180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9750,6 +9750,116 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>step-up-10k-milestone</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>N/A (Stats and Proof)</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>8</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/step-up-10k-2026-03-27/step-up-10k-milestone</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>10,000+ Copies Sold milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>step-up-3-stages</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>N/A (Stats and Proof)</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>8</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/step-up-10k-2026-03-27/step-up-3-stages</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Pinterest (no boards)</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>3 Steps to Deal with Difficult People</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel log - Topic 1 done
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K180"/>
+  <dimension ref="A1:K183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9860,6 +9860,171 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>build-relationships-first</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>N/A - researched topic</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>8</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/first-year-principal-2026-03-27/build-relationships-first</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Topic 1 of 4 this session</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>avoid-common-mistakes</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>N/A - researched topic</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>8</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/first-year-principal-2026-03-27/avoid-common-mistakes</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Topic 1 of 4 this session</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>lead-instruction-with-confidence</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>N/A - researched topic</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>8</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/first-year-principal-2026-03-27/lead-instruction-with-confidence</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Certified Working Genius Facilitator | Author</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Topic 1 of 4 this session</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx — Topic 3 talented-individually-dysfunctional
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K186"/>
+  <dimension ref="A1:K189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10190,6 +10190,171 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>signs-of-team-dysfunction</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>N/A - pain point</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>9</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/talented-individually-dysfunctional-2026-03-27/signs-of-team-dysfunction</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Topic 3 of 4 this session</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>root-causes-team-dysfunction</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>N/A - pain point</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>7</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/talented-individually-dysfunctional-2026-03-27/root-causes-team-dysfunction</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Topic 3 of 4 this session</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>N/A - pain point</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>8</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/talented-individually-dysfunctional-2026-03-27/fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Topic 3 of 4 this session</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx — Topic 4 coaching-for-leaders
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K189"/>
+  <dimension ref="A1:K192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10355,6 +10355,171 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>why-listen-coaching-for-leaders</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>N/A - podcast rec</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>7</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/coaching-for-leaders-podcast-2026-03-27/why-listen-coaching-for-leaders</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Topic 4 of 4 this session</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>best-episodes-coaching-for-leaders</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>N/A - podcast rec</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>8</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/coaching-for-leaders-podcast-2026-03-27/best-episodes-coaching-for-leaders</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Topic 4 of 4 this session</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>lessons-from-coaching-for-leaders</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>N/A - podcast rec</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>7</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/coaching-for-leaders-podcast-2026-03-27/lessons-from-coaching-for-leaders</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>No (Pinterest skipped)</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Topic 4 of 4 this session</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel-log.xlsx - Topic 1 Ian Cumming testimonial
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K192"/>
+  <dimension ref="A1:K194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10520,6 +10520,106 @@
         </is>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Ian Cumming Testimonial</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>10</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/ian-cumming-testimonial-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>YouTube (queue full)</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Leadership Coach | Author</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Testimonial carousel</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>What Great Coaching Looks Like</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>8</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/great-coaching-2026-03-27</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>YouTube (queue full)</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Leadership Coach | Author</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Coaching principles carousel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel log - Step Up or Step Out
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K196"/>
+  <dimension ref="A1:K199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10720,6 +10720,129 @@
         </is>
       </c>
     </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>step-up-step-out-overview</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>8</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>step-up-step-out-2026-03-28/step-up-step-out-overview</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>LI,FB,IG,Threads,X,GBP,TikTok,YT,Bluesky</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I197" t="b">
+        <v>1</v>
+      </c>
+      <c r="J197" t="b">
+        <v>1</v>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Framework overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>step-up-step-out-3-stages</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>8</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>step-up-step-out-2026-03-28/step-up-step-out-3-stages</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>LI,FB,IG,Threads,X,GBP,TikTok,YT,Bluesky</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I198" t="b">
+        <v>1</v>
+      </c>
+      <c r="J198" t="b">
+        <v>1</v>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>3 stages deep dive</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>step-up-step-out-apply</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>8</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>step-up-step-out-2026-03-28/step-up-step-out-apply</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>LI,FB,IG,Threads,X,GBP,TikTok,YT,Bluesky</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Author | Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="I199" t="b">
+        <v>1</v>
+      </c>
+      <c r="J199" t="b">
+        <v>1</v>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>5 practical actions</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update carousel log - Topic 1 GLS Podcast
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/carousel-log.xlsx
+++ b/data/carousel-workflow/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K208"/>
+  <dimension ref="A1:K211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11146,6 +11146,153 @@
         </is>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>gls-podcast</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>N/A - Podcast Recommendation</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>8</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/gls-podcast-2026-03-29</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>YouTube (queue full)</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>gls-podcast-guests</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>N/A - Podcast Recommendation</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>10</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/gls-podcast-guests-2026-03-29</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>YouTube (queue full)</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>gls-podcast-themes</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>N/A - Podcast Recommendation</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>7</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/carousels/gls-podcast-themes-2026-03-29</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>YouTube (queue full)</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Leadership Team Facilitator | Keynote Speaker | Author</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>